<commit_message>
updated architecture parsing dictionary, include ggplot of excel data
</commit_message>
<xml_diff>
--- a/Deep_Learning/Model_Optimization.xlsx
+++ b/Deep_Learning/Model_Optimization.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Full_Name</t>
   </si>
@@ -28,43 +28,67 @@
     <t>max_filters</t>
   </si>
   <si>
+    <t>atrous_blocks</t>
+  </si>
+  <si>
+    <t>atrous_rate</t>
+  </si>
+  <si>
+    <t>max_atrous_blocks</t>
+  </si>
+  <si>
+    <t>min_lr</t>
+  </si>
+  <si>
+    <t>max_lr</t>
+  </si>
+  <si>
+    <t>step_size_factor</t>
+  </si>
+  <si>
+    <t>num_cycles</t>
+  </si>
+  <si>
     <t>val_loss</t>
   </si>
   <si>
     <t>val_dice_coef_3D</t>
   </si>
   <si>
-    <t>4layers8filters16max_filters</t>
-  </si>
-  <si>
-    <t>4layers8filters32max_filters</t>
-  </si>
-  <si>
-    <t>4layers16filters32max_filters</t>
-  </si>
-  <si>
-    <t>5layers8filters16max_filters</t>
-  </si>
-  <si>
-    <t>5layers8filters32max_filters</t>
-  </si>
-  <si>
-    <t>5layers16filters32max_filters</t>
-  </si>
-  <si>
-    <t>3layers8filters16max_filters</t>
-  </si>
-  <si>
-    <t>3layers8filters32max_filters</t>
-  </si>
-  <si>
-    <t>3layers16filters32max_filters</t>
-  </si>
-  <si>
-    <t>inf</t>
-  </si>
-  <si>
-    <t>-inf</t>
+    <t>1layers8filters32max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers8filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers16filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers8filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers16filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers8filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers16filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>6layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
 </sst>
 </file>
@@ -422,10 +446,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -444,73 +468,157 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>8</v>
       </c>
       <c r="D2">
+        <v>32</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>2e-07</v>
+      </c>
+      <c r="I2">
+        <v>0.0007</v>
+      </c>
+      <c r="J2">
+        <v>8</v>
+      </c>
+      <c r="K2">
+        <v>5</v>
+      </c>
+      <c r="L2">
+        <v>0.01146829500794411</v>
+      </c>
+      <c r="M2">
+        <v>0.297448992729187</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>8</v>
+      </c>
+      <c r="D3">
         <v>16</v>
       </c>
-      <c r="E2">
-        <v>0.008781103417277336</v>
-      </c>
-      <c r="F2">
-        <v>0.3208378255367279</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>8</v>
-      </c>
-      <c r="D3">
-        <v>32</v>
-      </c>
       <c r="E3">
-        <v>0.008366866037249565</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>0.3436899781227112</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>3</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>2e-07</v>
+      </c>
+      <c r="I3">
+        <v>0.0007</v>
+      </c>
+      <c r="J3">
+        <v>8</v>
+      </c>
+      <c r="K3">
+        <v>5</v>
+      </c>
+      <c r="L3">
+        <v>0.01780537143349648</v>
+      </c>
+      <c r="M3">
+        <v>0.1700499802827835</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
       <c r="C4">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D4">
         <v>32</v>
       </c>
       <c r="E4">
-        <v>0.007578491698950529</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>0.3731243908405304</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>2e-07</v>
+      </c>
+      <c r="I4">
+        <v>0.0007</v>
+      </c>
+      <c r="J4">
+        <v>8</v>
+      </c>
+      <c r="K4">
+        <v>5</v>
+      </c>
+      <c r="L4">
+        <v>0.008729113265872002</v>
+      </c>
+      <c r="M4">
+        <v>0.3363664150238037</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B5">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C5">
         <v>8</v>
@@ -519,58 +627,121 @@
         <v>16</v>
       </c>
       <c r="E5">
-        <v>0.007827567867934704</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>0.3285523951053619</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>2e-07</v>
+      </c>
+      <c r="I5">
+        <v>0.0007</v>
+      </c>
+      <c r="J5">
+        <v>8</v>
+      </c>
+      <c r="K5">
+        <v>5</v>
+      </c>
+      <c r="L5">
+        <v>0.007943892851471901</v>
+      </c>
+      <c r="M5">
+        <v>0.3433967530727386</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="B6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D6">
         <v>32</v>
       </c>
       <c r="E6">
-        <v>0.006871452089399099</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>0.3513638079166412</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>1</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>2e-07</v>
+      </c>
+      <c r="I6">
+        <v>0.0007</v>
+      </c>
+      <c r="J6">
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>5</v>
+      </c>
+      <c r="L6">
+        <v>0.008382503874599934</v>
+      </c>
+      <c r="M6">
+        <v>0.3691894114017487</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B7">
         <v>5</v>
       </c>
       <c r="C7">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D7">
         <v>32</v>
       </c>
-      <c r="E7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>2e-07</v>
+      </c>
+      <c r="I7">
+        <v>0.0007</v>
+      </c>
+      <c r="J7">
+        <v>8</v>
+      </c>
+      <c r="K7">
+        <v>5</v>
+      </c>
+      <c r="L7">
+        <v>0.01328015048056841</v>
+      </c>
+      <c r="M7">
+        <v>0.09656653553247452</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C8">
         <v>8</v>
@@ -579,50 +750,236 @@
         <v>16</v>
       </c>
       <c r="E8">
-        <v>0.0101887471973896</v>
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>0.3121433854103088</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>2e-07</v>
+      </c>
+      <c r="I8">
+        <v>0.0007</v>
+      </c>
+      <c r="J8">
+        <v>8</v>
+      </c>
+      <c r="K8">
+        <v>5</v>
+      </c>
+      <c r="L8">
+        <v>0.006774149369448423</v>
+      </c>
+      <c r="M8">
+        <v>0.3602822124958038</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C9">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D9">
         <v>32</v>
       </c>
       <c r="E9">
-        <v>0.009529657661914825</v>
+        <v>1</v>
       </c>
       <c r="F9">
-        <v>0.338685542345047</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>2e-07</v>
+      </c>
+      <c r="I9">
+        <v>0.0007</v>
+      </c>
+      <c r="J9">
+        <v>8</v>
+      </c>
+      <c r="K9">
+        <v>5</v>
+      </c>
+      <c r="L9">
+        <v>0.01461964100599289</v>
+      </c>
+      <c r="M9">
+        <v>0.09296708554029465</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B10">
         <v>3</v>
       </c>
       <c r="C10">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D10">
         <v>32</v>
       </c>
       <c r="E10">
-        <v>0.008786829188466072</v>
+        <v>1</v>
       </c>
       <c r="F10">
-        <v>0.373685210943222</v>
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>2e-07</v>
+      </c>
+      <c r="I10">
+        <v>0.0007</v>
+      </c>
+      <c r="J10">
+        <v>8</v>
+      </c>
+      <c r="K10">
+        <v>5</v>
+      </c>
+      <c r="L10">
+        <v>0.01031966041773558</v>
+      </c>
+      <c r="M10">
+        <v>0.3306339383125305</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13">
+      <c r="A11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>8</v>
+      </c>
+      <c r="D11">
+        <v>16</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>2e-07</v>
+      </c>
+      <c r="I11">
+        <v>0.0007</v>
+      </c>
+      <c r="J11">
+        <v>8</v>
+      </c>
+      <c r="K11">
+        <v>5</v>
+      </c>
+      <c r="L11">
+        <v>0.009471160359680653</v>
+      </c>
+      <c r="M11">
+        <v>0.3350515365600586</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12">
+        <v>16</v>
+      </c>
+      <c r="D12">
+        <v>32</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>2e-07</v>
+      </c>
+      <c r="I12">
+        <v>0.0007</v>
+      </c>
+      <c r="J12">
+        <v>8</v>
+      </c>
+      <c r="K12">
+        <v>5</v>
+      </c>
+      <c r="L12">
+        <v>0.008939820341765881</v>
+      </c>
+      <c r="M12">
+        <v>0.35904461145401</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13">
+        <v>6</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13">
+        <v>16</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>2e-07</v>
+      </c>
+      <c r="I13">
+        <v>0.0007</v>
+      </c>
+      <c r="J13">
+        <v>8</v>
+      </c>
+      <c r="K13">
+        <v>5</v>
+      </c>
+      <c r="L13">
+        <v>0.005876542069017887</v>
+      </c>
+      <c r="M13">
+        <v>0.3382485806941986</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update find learning rate, also with ordered dict
</commit_message>
<xml_diff>
--- a/Deep_Learning/Model_Optimization.xlsx
+++ b/Deep_Learning/Model_Optimization.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>Full_Name</t>
   </si>
@@ -55,40 +55,115 @@
     <t>val_dice_coef_3D</t>
   </si>
   <si>
+    <t>7layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>7layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>7layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers8filters16max_filters1atrous_blocks5atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
     <t>1layers8filters32max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
     <t>1layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
-    <t>4layers8filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+    <t>8layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>8layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>8layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers8filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers16filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
     <t>4layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
-    <t>4layers16filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>5layers8filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+    <t>4layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers8filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers16filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
     <t>5layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
-    <t>5layers16filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>3layers8filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+    <t>5layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers8filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers16filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
     <t>3layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
-    <t>3layers16filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+    <t>3layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>6layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
   <si>
     <t>6layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>6layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
   </si>
 </sst>
 </file>
@@ -446,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -495,19 +570,19 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>8</v>
       </c>
       <c r="D2">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -525,10 +600,10 @@
         <v>5</v>
       </c>
       <c r="L2">
-        <v>0.01146829500794411</v>
+        <v>0.03072374500334263</v>
       </c>
       <c r="M2">
-        <v>0.297448992729187</v>
+        <v>0.09610175341367722</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -536,7 +611,7 @@
         <v>14</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C3">
         <v>8</v>
@@ -548,7 +623,7 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -566,10 +641,10 @@
         <v>5</v>
       </c>
       <c r="L3">
-        <v>0.01780537143349648</v>
+        <v>0.01252910308539867</v>
       </c>
       <c r="M3">
-        <v>0.1700499802827835</v>
+        <v>0.2924409806728363</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -577,19 +652,19 @@
         <v>15</v>
       </c>
       <c r="B4">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C4">
         <v>8</v>
       </c>
       <c r="D4">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G4">
         <v>1</v>
@@ -607,10 +682,10 @@
         <v>5</v>
       </c>
       <c r="L4">
-        <v>0.008729113265872002</v>
+        <v>0.02636530622839928</v>
       </c>
       <c r="M4">
-        <v>0.3363664150238037</v>
+        <v>0.04230921342968941</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -618,7 +693,7 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C5">
         <v>8</v>
@@ -630,7 +705,7 @@
         <v>1</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -648,10 +723,10 @@
         <v>5</v>
       </c>
       <c r="L5">
-        <v>0.007943892851471901</v>
+        <v>0.01390550844371319</v>
       </c>
       <c r="M5">
-        <v>0.3433967530727386</v>
+        <v>0.2876830399036407</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -659,20 +734,20 @@
         <v>17</v>
       </c>
       <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>16</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
         <v>4</v>
       </c>
-      <c r="C6">
-        <v>16</v>
-      </c>
-      <c r="D6">
-        <v>32</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
       <c r="G6">
         <v>1</v>
       </c>
@@ -689,10 +764,10 @@
         <v>5</v>
       </c>
       <c r="L6">
-        <v>0.008382503874599934</v>
+        <v>0.0152658075094223</v>
       </c>
       <c r="M6">
-        <v>0.3691894114017487</v>
+        <v>0.238678365945816</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -700,19 +775,19 @@
         <v>18</v>
       </c>
       <c r="B7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C7">
         <v>8</v>
       </c>
       <c r="D7">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7">
         <v>1</v>
@@ -730,10 +805,10 @@
         <v>5</v>
       </c>
       <c r="L7">
-        <v>0.01328015048056841</v>
+        <v>0.01298687607049942</v>
       </c>
       <c r="M7">
-        <v>0.09656653553247452</v>
+        <v>0.266437828540802</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -741,7 +816,7 @@
         <v>19</v>
       </c>
       <c r="B8">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C8">
         <v>8</v>
@@ -771,10 +846,10 @@
         <v>5</v>
       </c>
       <c r="L8">
-        <v>0.006774149369448423</v>
+        <v>0.01546592731028795</v>
       </c>
       <c r="M8">
-        <v>0.3602822124958038</v>
+        <v>0.1882520914077759</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -782,10 +857,10 @@
         <v>20</v>
       </c>
       <c r="B9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C9">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D9">
         <v>32</v>
@@ -794,7 +869,7 @@
         <v>1</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -812,10 +887,10 @@
         <v>5</v>
       </c>
       <c r="L9">
-        <v>0.01461964100599289</v>
+        <v>0.01146829500794411</v>
       </c>
       <c r="M9">
-        <v>0.09296708554029465</v>
+        <v>0.297448992729187</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -823,20 +898,20 @@
         <v>21</v>
       </c>
       <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10">
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>16</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
         <v>3</v>
       </c>
-      <c r="C10">
-        <v>8</v>
-      </c>
-      <c r="D10">
-        <v>32</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
       <c r="G10">
         <v>1</v>
       </c>
@@ -853,10 +928,10 @@
         <v>5</v>
       </c>
       <c r="L10">
-        <v>0.01031966041773558</v>
+        <v>0.01496024709194899</v>
       </c>
       <c r="M10">
-        <v>0.3306339383125305</v>
+        <v>0.2419810593128204</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -864,7 +939,7 @@
         <v>22</v>
       </c>
       <c r="B11">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C11">
         <v>8</v>
@@ -876,7 +951,7 @@
         <v>1</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -894,10 +969,10 @@
         <v>5</v>
       </c>
       <c r="L11">
-        <v>0.009471160359680653</v>
+        <v>0.01256441697478294</v>
       </c>
       <c r="M11">
-        <v>0.3350515365600586</v>
+        <v>0.3060401380062103</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -905,13 +980,13 @@
         <v>23</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C12">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="D12">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -935,10 +1010,10 @@
         <v>5</v>
       </c>
       <c r="L12">
-        <v>0.008939820341765881</v>
+        <v>0.01763521134853363</v>
       </c>
       <c r="M12">
-        <v>0.35904461145401</v>
+        <v>0.1320220082998276</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -946,40 +1021,1065 @@
         <v>24</v>
       </c>
       <c r="B13">
+        <v>8</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13">
+        <v>16</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>2e-07</v>
+      </c>
+      <c r="I13">
+        <v>0.0007</v>
+      </c>
+      <c r="J13">
+        <v>8</v>
+      </c>
+      <c r="K13">
+        <v>5</v>
+      </c>
+      <c r="L13">
+        <v>0.02592094987630844</v>
+      </c>
+      <c r="M13">
+        <v>0.04257644340395927</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14">
+        <v>4</v>
+      </c>
+      <c r="C14">
+        <v>8</v>
+      </c>
+      <c r="D14">
+        <v>16</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>4</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>2e-07</v>
+      </c>
+      <c r="I14">
+        <v>0.0007</v>
+      </c>
+      <c r="J14">
+        <v>8</v>
+      </c>
+      <c r="K14">
+        <v>5</v>
+      </c>
+      <c r="L14">
+        <v>0.0297101978212595</v>
+      </c>
+      <c r="M14">
+        <v>0.03271352127194405</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15">
+        <v>8</v>
+      </c>
+      <c r="D15">
+        <v>32</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>2e-07</v>
+      </c>
+      <c r="I15">
+        <v>0.0007</v>
+      </c>
+      <c r="J15">
+        <v>8</v>
+      </c>
+      <c r="K15">
+        <v>5</v>
+      </c>
+      <c r="L15">
+        <v>0.008729113265872002</v>
+      </c>
+      <c r="M15">
+        <v>0.3363664150238037</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13">
+      <c r="A16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16">
+        <v>4</v>
+      </c>
+      <c r="C16">
+        <v>8</v>
+      </c>
+      <c r="D16">
+        <v>16</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>2e-07</v>
+      </c>
+      <c r="I16">
+        <v>0.0007</v>
+      </c>
+      <c r="J16">
+        <v>8</v>
+      </c>
+      <c r="K16">
+        <v>5</v>
+      </c>
+      <c r="L16">
+        <v>0.007943892851471901</v>
+      </c>
+      <c r="M16">
+        <v>0.3514969944953918</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13">
+      <c r="A17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+      <c r="D17">
+        <v>32</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>2e-07</v>
+      </c>
+      <c r="I17">
+        <v>0.0007</v>
+      </c>
+      <c r="J17">
+        <v>8</v>
+      </c>
+      <c r="K17">
+        <v>5</v>
+      </c>
+      <c r="L17">
+        <v>0.008382503874599934</v>
+      </c>
+      <c r="M17">
+        <v>0.3691894114017487</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13">
+      <c r="A18" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>8</v>
+      </c>
+      <c r="D18">
+        <v>16</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>2e-07</v>
+      </c>
+      <c r="I18">
+        <v>0.0007</v>
+      </c>
+      <c r="J18">
+        <v>8</v>
+      </c>
+      <c r="K18">
+        <v>5</v>
+      </c>
+      <c r="L18">
+        <v>0.01297671347856522</v>
+      </c>
+      <c r="M18">
+        <v>0.289603978395462</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13">
+      <c r="A19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19">
+        <v>4</v>
+      </c>
+      <c r="C19">
+        <v>8</v>
+      </c>
+      <c r="D19">
+        <v>16</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>3</v>
+      </c>
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>2e-07</v>
+      </c>
+      <c r="I19">
+        <v>0.0007</v>
+      </c>
+      <c r="J19">
+        <v>8</v>
+      </c>
+      <c r="K19">
+        <v>5</v>
+      </c>
+      <c r="L19">
+        <v>0.0260687954723835</v>
+      </c>
+      <c r="M19">
+        <v>0.04598050564527512</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13">
+      <c r="A20" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20">
+        <v>5</v>
+      </c>
+      <c r="C20">
+        <v>8</v>
+      </c>
+      <c r="D20">
+        <v>16</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>4</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>2e-07</v>
+      </c>
+      <c r="I20">
+        <v>0.0007</v>
+      </c>
+      <c r="J20">
+        <v>8</v>
+      </c>
+      <c r="K20">
+        <v>5</v>
+      </c>
+      <c r="L20">
+        <v>0.0360008031129837</v>
+      </c>
+      <c r="M20">
+        <v>0.02795693278312683</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13">
+      <c r="A21" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21">
+        <v>5</v>
+      </c>
+      <c r="C21">
+        <v>8</v>
+      </c>
+      <c r="D21">
+        <v>32</v>
+      </c>
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>2e-07</v>
+      </c>
+      <c r="I21">
+        <v>0.0007</v>
+      </c>
+      <c r="J21">
+        <v>8</v>
+      </c>
+      <c r="K21">
+        <v>5</v>
+      </c>
+      <c r="L21">
+        <v>0.01328015048056841</v>
+      </c>
+      <c r="M21">
+        <v>0.09656653553247452</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13">
+      <c r="A22" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22">
+        <v>5</v>
+      </c>
+      <c r="C22">
+        <v>8</v>
+      </c>
+      <c r="D22">
+        <v>16</v>
+      </c>
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
+        <v>2</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>2e-07</v>
+      </c>
+      <c r="I22">
+        <v>0.0007</v>
+      </c>
+      <c r="J22">
+        <v>8</v>
+      </c>
+      <c r="K22">
+        <v>5</v>
+      </c>
+      <c r="L22">
+        <v>0.006774149369448423</v>
+      </c>
+      <c r="M22">
+        <v>0.3780486583709717</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13">
+      <c r="A23" t="s">
+        <v>34</v>
+      </c>
+      <c r="B23">
+        <v>5</v>
+      </c>
+      <c r="C23">
+        <v>16</v>
+      </c>
+      <c r="D23">
+        <v>32</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
+        <v>2</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>2e-07</v>
+      </c>
+      <c r="I23">
+        <v>0.0007</v>
+      </c>
+      <c r="J23">
+        <v>8</v>
+      </c>
+      <c r="K23">
+        <v>5</v>
+      </c>
+      <c r="L23">
+        <v>0.01461964100599289</v>
+      </c>
+      <c r="M23">
+        <v>0.09296708554029465</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13">
+      <c r="A24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24">
+        <v>5</v>
+      </c>
+      <c r="C24">
+        <v>8</v>
+      </c>
+      <c r="D24">
+        <v>16</v>
+      </c>
+      <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>2e-07</v>
+      </c>
+      <c r="I24">
+        <v>0.0007</v>
+      </c>
+      <c r="J24">
+        <v>8</v>
+      </c>
+      <c r="K24">
+        <v>5</v>
+      </c>
+      <c r="L24">
+        <v>0.01157489139586687</v>
+      </c>
+      <c r="M24">
+        <v>0.3093194663524628</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25">
+        <v>5</v>
+      </c>
+      <c r="C25">
+        <v>8</v>
+      </c>
+      <c r="D25">
+        <v>16</v>
+      </c>
+      <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
+        <v>3</v>
+      </c>
+      <c r="G25">
+        <v>1</v>
+      </c>
+      <c r="H25">
+        <v>2e-07</v>
+      </c>
+      <c r="I25">
+        <v>0.0007</v>
+      </c>
+      <c r="J25">
+        <v>8</v>
+      </c>
+      <c r="K25">
+        <v>5</v>
+      </c>
+      <c r="L25">
+        <v>0.02652654238045216</v>
+      </c>
+      <c r="M25">
+        <v>0.05044718086719513</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13">
+      <c r="A26" t="s">
+        <v>37</v>
+      </c>
+      <c r="B26">
+        <v>3</v>
+      </c>
+      <c r="C26">
+        <v>8</v>
+      </c>
+      <c r="D26">
+        <v>16</v>
+      </c>
+      <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
+        <v>4</v>
+      </c>
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>2e-07</v>
+      </c>
+      <c r="I26">
+        <v>0.0007</v>
+      </c>
+      <c r="J26">
+        <v>8</v>
+      </c>
+      <c r="K26">
+        <v>5</v>
+      </c>
+      <c r="L26">
+        <v>0.0144530413672328</v>
+      </c>
+      <c r="M26">
+        <v>0.2646083831787109</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13">
+      <c r="A27" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+      <c r="C27">
+        <v>8</v>
+      </c>
+      <c r="D27">
+        <v>32</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
+        <v>2</v>
+      </c>
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>2e-07</v>
+      </c>
+      <c r="I27">
+        <v>0.0007</v>
+      </c>
+      <c r="J27">
+        <v>8</v>
+      </c>
+      <c r="K27">
+        <v>5</v>
+      </c>
+      <c r="L27">
+        <v>0.01031966041773558</v>
+      </c>
+      <c r="M27">
+        <v>0.3306339383125305</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13">
+      <c r="A28" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28">
+        <v>8</v>
+      </c>
+      <c r="D28">
+        <v>16</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28">
+        <v>2</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28">
+        <v>2e-07</v>
+      </c>
+      <c r="I28">
+        <v>0.0007</v>
+      </c>
+      <c r="J28">
+        <v>8</v>
+      </c>
+      <c r="K28">
+        <v>5</v>
+      </c>
+      <c r="L28">
+        <v>0.009471160359680653</v>
+      </c>
+      <c r="M28">
+        <v>0.3517069518566132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
+      <c r="A29" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+      <c r="C29">
+        <v>16</v>
+      </c>
+      <c r="D29">
+        <v>32</v>
+      </c>
+      <c r="E29">
+        <v>1</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
+        <v>2e-07</v>
+      </c>
+      <c r="I29">
+        <v>0.0007</v>
+      </c>
+      <c r="J29">
+        <v>8</v>
+      </c>
+      <c r="K29">
+        <v>5</v>
+      </c>
+      <c r="L29">
+        <v>0.008939820341765881</v>
+      </c>
+      <c r="M29">
+        <v>0.35904461145401</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13">
+      <c r="A30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+      <c r="C30">
+        <v>8</v>
+      </c>
+      <c r="D30">
+        <v>16</v>
+      </c>
+      <c r="E30">
+        <v>1</v>
+      </c>
+      <c r="F30">
+        <v>1</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
+        <v>2e-07</v>
+      </c>
+      <c r="I30">
+        <v>0.0007</v>
+      </c>
+      <c r="J30">
+        <v>8</v>
+      </c>
+      <c r="K30">
+        <v>5</v>
+      </c>
+      <c r="L30">
+        <v>0.01335400622338057</v>
+      </c>
+      <c r="M30">
+        <v>0.2640894949436188</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13">
+      <c r="A31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31">
+        <v>3</v>
+      </c>
+      <c r="C31">
+        <v>8</v>
+      </c>
+      <c r="D31">
+        <v>16</v>
+      </c>
+      <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
+        <v>3</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
+      </c>
+      <c r="H31">
+        <v>2e-07</v>
+      </c>
+      <c r="I31">
+        <v>0.0007</v>
+      </c>
+      <c r="J31">
+        <v>8</v>
+      </c>
+      <c r="K31">
+        <v>5</v>
+      </c>
+      <c r="L31">
+        <v>0.02298250235617161</v>
+      </c>
+      <c r="M31">
+        <v>0.08047252893447876</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" t="s">
+        <v>43</v>
+      </c>
+      <c r="B32">
         <v>6</v>
       </c>
-      <c r="C13">
-        <v>8</v>
-      </c>
-      <c r="D13">
-        <v>16</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-      <c r="H13">
-        <v>2e-07</v>
-      </c>
-      <c r="I13">
-        <v>0.0007</v>
-      </c>
-      <c r="J13">
-        <v>8</v>
-      </c>
-      <c r="K13">
-        <v>5</v>
-      </c>
-      <c r="L13">
+      <c r="C32">
+        <v>8</v>
+      </c>
+      <c r="D32">
+        <v>16</v>
+      </c>
+      <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
+        <v>2</v>
+      </c>
+      <c r="G32">
+        <v>1</v>
+      </c>
+      <c r="H32">
+        <v>2e-07</v>
+      </c>
+      <c r="I32">
+        <v>0.0007</v>
+      </c>
+      <c r="J32">
+        <v>8</v>
+      </c>
+      <c r="K32">
+        <v>5</v>
+      </c>
+      <c r="L32">
         <v>0.005876542069017887</v>
       </c>
-      <c r="M13">
-        <v>0.3382485806941986</v>
+      <c r="M32">
+        <v>0.3449607789516449</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13">
+      <c r="A33" t="s">
+        <v>44</v>
+      </c>
+      <c r="B33">
+        <v>6</v>
+      </c>
+      <c r="C33">
+        <v>8</v>
+      </c>
+      <c r="D33">
+        <v>16</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
+        <v>1</v>
+      </c>
+      <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="H33">
+        <v>2e-07</v>
+      </c>
+      <c r="I33">
+        <v>0.0007</v>
+      </c>
+      <c r="J33">
+        <v>8</v>
+      </c>
+      <c r="K33">
+        <v>5</v>
+      </c>
+      <c r="L33">
+        <v>0.01197956781834364</v>
+      </c>
+      <c r="M33">
+        <v>0.2813169360160828</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13">
+      <c r="A34" t="s">
+        <v>45</v>
+      </c>
+      <c r="B34">
+        <v>6</v>
+      </c>
+      <c r="C34">
+        <v>8</v>
+      </c>
+      <c r="D34">
+        <v>16</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
+        <v>3</v>
+      </c>
+      <c r="G34">
+        <v>1</v>
+      </c>
+      <c r="H34">
+        <v>2e-07</v>
+      </c>
+      <c r="I34">
+        <v>0.0007</v>
+      </c>
+      <c r="J34">
+        <v>8</v>
+      </c>
+      <c r="K34">
+        <v>5</v>
+      </c>
+      <c r="L34">
+        <v>0.01171945314854383</v>
+      </c>
+      <c r="M34">
+        <v>0.3067871332168579</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13">
+      <c r="A35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>8</v>
+      </c>
+      <c r="D35">
+        <v>16</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
+        <v>4</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35">
+        <v>2e-07</v>
+      </c>
+      <c r="I35">
+        <v>0.0007</v>
+      </c>
+      <c r="J35">
+        <v>8</v>
+      </c>
+      <c r="K35">
+        <v>5</v>
+      </c>
+      <c r="L35">
+        <v>0.02075445093214512</v>
+      </c>
+      <c r="M35">
+        <v>0.1012341752648354</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13">
+      <c r="A36" t="s">
+        <v>47</v>
+      </c>
+      <c r="B36">
+        <v>2</v>
+      </c>
+      <c r="C36">
+        <v>8</v>
+      </c>
+      <c r="D36">
+        <v>16</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36">
+        <v>2e-07</v>
+      </c>
+      <c r="I36">
+        <v>0.0007</v>
+      </c>
+      <c r="J36">
+        <v>8</v>
+      </c>
+      <c r="K36">
+        <v>5</v>
+      </c>
+      <c r="L36">
+        <v>0.01198610290884972</v>
+      </c>
+      <c r="M36">
+        <v>0.2936770021915436</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13">
+      <c r="A37" t="s">
+        <v>48</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>8</v>
+      </c>
+      <c r="D37">
+        <v>16</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37">
+        <v>1</v>
+      </c>
+      <c r="G37">
+        <v>1</v>
+      </c>
+      <c r="H37">
+        <v>2e-07</v>
+      </c>
+      <c r="I37">
+        <v>0.0007</v>
+      </c>
+      <c r="J37">
+        <v>8</v>
+      </c>
+      <c r="K37">
+        <v>5</v>
+      </c>
+      <c r="L37">
+        <v>0.01439808961004019</v>
+      </c>
+      <c r="M37">
+        <v>0.2381373792886734</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13">
+      <c r="A38" t="s">
+        <v>49</v>
+      </c>
+      <c r="B38">
+        <v>2</v>
+      </c>
+      <c r="C38">
+        <v>8</v>
+      </c>
+      <c r="D38">
+        <v>16</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38">
+        <v>3</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38">
+        <v>2e-07</v>
+      </c>
+      <c r="I38">
+        <v>0.0007</v>
+      </c>
+      <c r="J38">
+        <v>8</v>
+      </c>
+      <c r="K38">
+        <v>5</v>
+      </c>
+      <c r="L38">
+        <v>0.01031064987182617</v>
+      </c>
+      <c r="M38">
+        <v>0.3455671370029449</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
improved plotting with plot9 ggplot, added figures
</commit_message>
<xml_diff>
--- a/Deep_Learning/Model_Optimization.xlsx
+++ b/Deep_Learning/Model_Optimization.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>Full_Name</t>
   </si>
@@ -55,115 +55,130 @@
     <t>val_dice_coef_3D</t>
   </si>
   <si>
-    <t>7layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>7layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>7layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>1layers8filters16max_filters1atrous_blocks5atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>1layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>1layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>1layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>1layers8filters32max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>1layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>8layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>8layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>8layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>4layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>4layers8filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>4layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>4layers16filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>4layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>4layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>5layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>5layers8filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>5layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>5layers16filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>5layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>5layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>3layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>3layers8filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>3layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>3layers16filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>3layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>3layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>6layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>6layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>6layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>2layers8filters16max_filters1atrous_blocks4atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>2layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>2layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
-  </si>
-  <si>
-    <t>2layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-07min_lr0.0007max_lr8step_size_factor5num_cycles</t>
+    <t>7layers16filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks1e-06min_lr0.0001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>7layers32filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>7layers16filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks8e-07min_lr0.0001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>7layers32filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr7e-06max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers8filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks1e-05min_lr0.002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers16filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-06min_lr0.001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers32filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-06min_lr0.0002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers8filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks1e-05min_lr0.01max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers16filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks1e-05min_lr0.003max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers32filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks3e-06min_lr0.002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers8filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks1e-05min_lr0.0002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers16filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks2e-06min_lr0.00017max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>1layers32filters32max_filters1atrous_blocks3atrous_rate1max_atrous_blocks1e-06min_lr6e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>8layers16filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks6e-07min_lr4e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>8layers16filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks1e-06min_lr0.0001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>8layers32filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks6e-07min_lr2e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers16filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks1.8e-06min_lr0.0004max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers32filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks1e-06min_lr0.0002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers16filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks5e-06min_lr0.0002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers32filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks1e-06min_lr0.00015max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>4layers16filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks1e-06min_lr5e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers16filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-06min_lr0.00015max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers32filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr5e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers16filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks1.5e-06min_lr0.0002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers32filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr0.0002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>5layers16filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks1e-06min_lr0.0001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers16filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks1e-06min_lr0.0001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers32filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks5e-07min_lr7e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers16filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-06min_lr0.001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers32filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks1e-06min_lr0.00015max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers16filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks1e-06min_lr0.0008max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>3layers32filters32max_filters1atrous_blocks3atrous_rate1max_atrous_blocks1e-06min_lr2.5e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>6layers16filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks1e-06min_lr8e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>6layers32filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-07min_lr0.0001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>6layers16filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-06min_lr6e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>6layers32filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks2e-07min_lr3e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers16filters16max_filters1atrous_blocks2atrous_rate1max_atrous_blocks2e-06min_lr0.0001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers32filters32max_filters1atrous_blocks2atrous_rate1max_atrous_blocks1e-06min_lr0.00025max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers16filters16max_filters1atrous_blocks1atrous_rate1max_atrous_blocks6e-06min_lr0.0002max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers32filters32max_filters1atrous_blocks1atrous_rate1max_atrous_blocks1e-06min_lr0.001max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers16filters16max_filters1atrous_blocks3atrous_rate1max_atrous_blocks1.7e-06min_lr5e-05max_lr8step_size_factor5num_cycles</t>
+  </si>
+  <si>
+    <t>2layers32filters32max_filters1atrous_blocks3atrous_rate1max_atrous_blocks1e-06min_lr4e-05max_lr8step_size_factor5num_cycles</t>
   </si>
 </sst>
 </file>
@@ -521,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:13">
@@ -573,7 +588,7 @@
         <v>7</v>
       </c>
       <c r="C2">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D2">
         <v>16</v>
@@ -588,10 +603,10 @@
         <v>1</v>
       </c>
       <c r="H2">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I2">
-        <v>0.0007</v>
+        <v>0.0001</v>
       </c>
       <c r="J2">
         <v>8</v>
@@ -600,10 +615,10 @@
         <v>5</v>
       </c>
       <c r="L2">
-        <v>0.03072374500334263</v>
+        <v>0.01192688103765249</v>
       </c>
       <c r="M2">
-        <v>0.09610175341367722</v>
+        <v>0.2973805367946625</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -614,16 +629,16 @@
         <v>7</v>
       </c>
       <c r="C3">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D3">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -632,7 +647,7 @@
         <v>2e-07</v>
       </c>
       <c r="I3">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="J3">
         <v>8</v>
@@ -641,10 +656,10 @@
         <v>5</v>
       </c>
       <c r="L3">
-        <v>0.01252910308539867</v>
+        <v>0.01069515570998192</v>
       </c>
       <c r="M3">
-        <v>0.2924409806728363</v>
+        <v>0.3540820181369781</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -655,7 +670,7 @@
         <v>7</v>
       </c>
       <c r="C4">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D4">
         <v>16</v>
@@ -664,16 +679,16 @@
         <v>1</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
       <c r="H4">
-        <v>2e-07</v>
+        <v>8e-07</v>
       </c>
       <c r="I4">
-        <v>0.0007</v>
+        <v>0.0001</v>
       </c>
       <c r="J4">
         <v>8</v>
@@ -682,10 +697,10 @@
         <v>5</v>
       </c>
       <c r="L4">
-        <v>0.02636530622839928</v>
+        <v>0.01579839736223221</v>
       </c>
       <c r="M4">
-        <v>0.04230921342968941</v>
+        <v>0.2252430766820908</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -693,19 +708,19 @@
         <v>16</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C5">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D5">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -714,7 +729,7 @@
         <v>2e-07</v>
       </c>
       <c r="I5">
-        <v>0.0007</v>
+        <v>7e-06</v>
       </c>
       <c r="J5">
         <v>8</v>
@@ -723,10 +738,10 @@
         <v>5</v>
       </c>
       <c r="L5">
-        <v>0.01390550844371319</v>
+        <v>0.0230035912245512</v>
       </c>
       <c r="M5">
-        <v>0.2876830399036407</v>
+        <v>0.1652709096670151</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -746,16 +761,16 @@
         <v>1</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
       <c r="H6">
-        <v>2e-07</v>
+        <v>1e-05</v>
       </c>
       <c r="I6">
-        <v>0.0007</v>
+        <v>0.002</v>
       </c>
       <c r="J6">
         <v>8</v>
@@ -764,10 +779,10 @@
         <v>5</v>
       </c>
       <c r="L6">
-        <v>0.0152658075094223</v>
+        <v>0.01383414771407843</v>
       </c>
       <c r="M6">
-        <v>0.238678365945816</v>
+        <v>0.2462903559207916</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -778,7 +793,7 @@
         <v>1</v>
       </c>
       <c r="C7">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D7">
         <v>16</v>
@@ -793,10 +808,10 @@
         <v>1</v>
       </c>
       <c r="H7">
-        <v>2e-07</v>
+        <v>2e-06</v>
       </c>
       <c r="I7">
-        <v>0.0007</v>
+        <v>0.001</v>
       </c>
       <c r="J7">
         <v>8</v>
@@ -805,10 +820,10 @@
         <v>5</v>
       </c>
       <c r="L7">
-        <v>0.01298687607049942</v>
+        <v>0.01491123158484697</v>
       </c>
       <c r="M7">
-        <v>0.266437828540802</v>
+        <v>0.2240881472826004</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -819,25 +834,25 @@
         <v>1</v>
       </c>
       <c r="C8">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D8">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8">
-        <v>2e-07</v>
+        <v>2e-06</v>
       </c>
       <c r="I8">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="J8">
         <v>8</v>
@@ -846,10 +861,10 @@
         <v>5</v>
       </c>
       <c r="L8">
-        <v>0.01546592731028795</v>
+        <v>0.01531479321420193</v>
       </c>
       <c r="M8">
-        <v>0.1882520914077759</v>
+        <v>0.2149901837110519</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -863,22 +878,22 @@
         <v>8</v>
       </c>
       <c r="D9">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G9">
         <v>1</v>
       </c>
       <c r="H9">
-        <v>2e-07</v>
+        <v>1e-05</v>
       </c>
       <c r="I9">
-        <v>0.0007</v>
+        <v>0.01</v>
       </c>
       <c r="J9">
         <v>8</v>
@@ -887,10 +902,10 @@
         <v>5</v>
       </c>
       <c r="L9">
-        <v>0.01146829500794411</v>
+        <v>0.01564678363502026</v>
       </c>
       <c r="M9">
-        <v>0.297448992729187</v>
+        <v>0.1878472566604614</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -901,7 +916,7 @@
         <v>1</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D10">
         <v>16</v>
@@ -910,16 +925,16 @@
         <v>1</v>
       </c>
       <c r="F10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G10">
         <v>1</v>
       </c>
       <c r="H10">
-        <v>2e-07</v>
+        <v>1e-05</v>
       </c>
       <c r="I10">
-        <v>0.0007</v>
+        <v>0.003</v>
       </c>
       <c r="J10">
         <v>8</v>
@@ -928,10 +943,10 @@
         <v>5</v>
       </c>
       <c r="L10">
-        <v>0.01496024709194899</v>
+        <v>0.01578664220869541</v>
       </c>
       <c r="M10">
-        <v>0.2419810593128204</v>
+        <v>0.2078990191221237</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -939,28 +954,28 @@
         <v>22</v>
       </c>
       <c r="B11">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C11">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D11">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
       <c r="H11">
-        <v>2e-07</v>
+        <v>3e-06</v>
       </c>
       <c r="I11">
-        <v>0.0007</v>
+        <v>0.002</v>
       </c>
       <c r="J11">
         <v>8</v>
@@ -969,10 +984,10 @@
         <v>5</v>
       </c>
       <c r="L11">
-        <v>0.01256441697478294</v>
+        <v>0.01563869044184685</v>
       </c>
       <c r="M11">
-        <v>0.3060401380062103</v>
+        <v>0.1988261938095093</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -980,7 +995,7 @@
         <v>23</v>
       </c>
       <c r="B12">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C12">
         <v>8</v>
@@ -992,16 +1007,16 @@
         <v>1</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G12">
         <v>1</v>
       </c>
       <c r="H12">
-        <v>2e-07</v>
+        <v>1e-05</v>
       </c>
       <c r="I12">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="J12">
         <v>8</v>
@@ -1010,10 +1025,10 @@
         <v>5</v>
       </c>
       <c r="L12">
-        <v>0.01763521134853363</v>
+        <v>0.01966289430856705</v>
       </c>
       <c r="M12">
-        <v>0.1320220082998276</v>
+        <v>0.1412597149610519</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1021,10 +1036,10 @@
         <v>24</v>
       </c>
       <c r="B13">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C13">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D13">
         <v>16</v>
@@ -1039,10 +1054,10 @@
         <v>1</v>
       </c>
       <c r="H13">
-        <v>2e-07</v>
+        <v>2e-06</v>
       </c>
       <c r="I13">
-        <v>0.0007</v>
+        <v>0.00017</v>
       </c>
       <c r="J13">
         <v>8</v>
@@ -1051,10 +1066,10 @@
         <v>5</v>
       </c>
       <c r="L13">
-        <v>0.02592094987630844</v>
+        <v>0.01759837009012699</v>
       </c>
       <c r="M13">
-        <v>0.04257644340395927</v>
+        <v>0.1507639437913895</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1062,28 +1077,28 @@
         <v>25</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C14">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D14">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E14">
         <v>1</v>
       </c>
       <c r="F14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G14">
         <v>1</v>
       </c>
       <c r="H14">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I14">
-        <v>0.0007</v>
+        <v>6e-05</v>
       </c>
       <c r="J14">
         <v>8</v>
@@ -1092,10 +1107,10 @@
         <v>5</v>
       </c>
       <c r="L14">
-        <v>0.0297101978212595</v>
+        <v>0.01871275343000889</v>
       </c>
       <c r="M14">
-        <v>0.03271352127194405</v>
+        <v>0.1581901758909225</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -1103,13 +1118,13 @@
         <v>26</v>
       </c>
       <c r="B15">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C15">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D15">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -1121,10 +1136,10 @@
         <v>1</v>
       </c>
       <c r="H15">
-        <v>2e-07</v>
+        <v>6e-07</v>
       </c>
       <c r="I15">
-        <v>0.0007</v>
+        <v>4e-05</v>
       </c>
       <c r="J15">
         <v>8</v>
@@ -1133,10 +1148,10 @@
         <v>5</v>
       </c>
       <c r="L15">
-        <v>0.008729113265872002</v>
+        <v>0.01690562069416046</v>
       </c>
       <c r="M15">
-        <v>0.3363664150238037</v>
+        <v>0.2183466106653214</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -1144,10 +1159,10 @@
         <v>27</v>
       </c>
       <c r="B16">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C16">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D16">
         <v>16</v>
@@ -1156,16 +1171,16 @@
         <v>1</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
       <c r="H16">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I16">
-        <v>0.0007</v>
+        <v>0.0001</v>
       </c>
       <c r="J16">
         <v>8</v>
@@ -1174,10 +1189,10 @@
         <v>5</v>
       </c>
       <c r="L16">
-        <v>0.007943892851471901</v>
+        <v>0.01620516367256641</v>
       </c>
       <c r="M16">
-        <v>0.3514969944953918</v>
+        <v>0.2279257923364639</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1185,10 +1200,10 @@
         <v>28</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C17">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D17">
         <v>32</v>
@@ -1197,16 +1212,16 @@
         <v>1</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17">
         <v>1</v>
       </c>
       <c r="H17">
-        <v>2e-07</v>
+        <v>6e-07</v>
       </c>
       <c r="I17">
-        <v>0.0007</v>
+        <v>2e-05</v>
       </c>
       <c r="J17">
         <v>8</v>
@@ -1215,10 +1230,10 @@
         <v>5</v>
       </c>
       <c r="L17">
-        <v>0.008382503874599934</v>
+        <v>0.0195910632610321</v>
       </c>
       <c r="M17">
-        <v>0.3691894114017487</v>
+        <v>0.2124533653259277</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1229,7 +1244,7 @@
         <v>4</v>
       </c>
       <c r="C18">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D18">
         <v>16</v>
@@ -1238,16 +1253,16 @@
         <v>1</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18">
         <v>1</v>
       </c>
       <c r="H18">
-        <v>2e-07</v>
+        <v>1.8e-06</v>
       </c>
       <c r="I18">
-        <v>0.0007</v>
+        <v>0.0004</v>
       </c>
       <c r="J18">
         <v>8</v>
@@ -1256,10 +1271,10 @@
         <v>5</v>
       </c>
       <c r="L18">
-        <v>0.01297671347856522</v>
+        <v>0.01142287626862526</v>
       </c>
       <c r="M18">
-        <v>0.289603978395462</v>
+        <v>0.3158088326454163</v>
       </c>
     </row>
     <row r="19" spans="1:13">
@@ -1270,25 +1285,25 @@
         <v>4</v>
       </c>
       <c r="C19">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D19">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G19">
         <v>1</v>
       </c>
       <c r="H19">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I19">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="J19">
         <v>8</v>
@@ -1297,10 +1312,10 @@
         <v>5</v>
       </c>
       <c r="L19">
-        <v>0.0260687954723835</v>
+        <v>0.01067902892827988</v>
       </c>
       <c r="M19">
-        <v>0.04598050564527512</v>
+        <v>0.3374375700950623</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1308,10 +1323,10 @@
         <v>31</v>
       </c>
       <c r="B20">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C20">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D20">
         <v>16</v>
@@ -1320,16 +1335,16 @@
         <v>1</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G20">
         <v>1</v>
       </c>
       <c r="H20">
-        <v>2e-07</v>
+        <v>5e-06</v>
       </c>
       <c r="I20">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="J20">
         <v>8</v>
@@ -1338,10 +1353,10 @@
         <v>5</v>
       </c>
       <c r="L20">
-        <v>0.0360008031129837</v>
+        <v>0.0156412310898304</v>
       </c>
       <c r="M20">
-        <v>0.02795693278312683</v>
+        <v>0.2165517508983612</v>
       </c>
     </row>
     <row r="21" spans="1:13">
@@ -1349,10 +1364,10 @@
         <v>32</v>
       </c>
       <c r="B21">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C21">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D21">
         <v>32</v>
@@ -1361,16 +1376,16 @@
         <v>1</v>
       </c>
       <c r="F21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G21">
         <v>1</v>
       </c>
       <c r="H21">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I21">
-        <v>0.0007</v>
+        <v>0.00015</v>
       </c>
       <c r="J21">
         <v>8</v>
@@ -1379,10 +1394,10 @@
         <v>5</v>
       </c>
       <c r="L21">
-        <v>0.01328015048056841</v>
+        <v>0.01484843157231808</v>
       </c>
       <c r="M21">
-        <v>0.09656653553247452</v>
+        <v>0.2374653369188309</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1390,10 +1405,10 @@
         <v>33</v>
       </c>
       <c r="B22">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C22">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D22">
         <v>16</v>
@@ -1402,16 +1417,16 @@
         <v>1</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G22">
         <v>1</v>
       </c>
       <c r="H22">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I22">
-        <v>0.0007</v>
+        <v>5e-05</v>
       </c>
       <c r="J22">
         <v>8</v>
@@ -1420,10 +1435,10 @@
         <v>5</v>
       </c>
       <c r="L22">
-        <v>0.006774149369448423</v>
+        <v>0.01789148151874542</v>
       </c>
       <c r="M22">
-        <v>0.3780486583709717</v>
+        <v>0.1609459668397903</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1437,7 +1452,7 @@
         <v>16</v>
       </c>
       <c r="D23">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -1449,10 +1464,10 @@
         <v>1</v>
       </c>
       <c r="H23">
-        <v>2e-07</v>
+        <v>2e-06</v>
       </c>
       <c r="I23">
-        <v>0.0007</v>
+        <v>0.00015</v>
       </c>
       <c r="J23">
         <v>8</v>
@@ -1461,10 +1476,10 @@
         <v>5</v>
       </c>
       <c r="L23">
-        <v>0.01461964100599289</v>
+        <v>0.01326036639511585</v>
       </c>
       <c r="M23">
-        <v>0.09296708554029465</v>
+        <v>0.2676254212856293</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -1475,16 +1490,16 @@
         <v>5</v>
       </c>
       <c r="C24">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D24">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -1493,7 +1508,7 @@
         <v>2e-07</v>
       </c>
       <c r="I24">
-        <v>0.0007</v>
+        <v>5e-05</v>
       </c>
       <c r="J24">
         <v>8</v>
@@ -1502,10 +1517,10 @@
         <v>5</v>
       </c>
       <c r="L24">
-        <v>0.01157489139586687</v>
+        <v>0.01356085110455751</v>
       </c>
       <c r="M24">
-        <v>0.3093194663524628</v>
+        <v>0.2645507454872131</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -1516,7 +1531,7 @@
         <v>5</v>
       </c>
       <c r="C25">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D25">
         <v>16</v>
@@ -1525,16 +1540,16 @@
         <v>1</v>
       </c>
       <c r="F25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G25">
         <v>1</v>
       </c>
       <c r="H25">
-        <v>2e-07</v>
+        <v>1.5e-06</v>
       </c>
       <c r="I25">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="J25">
         <v>8</v>
@@ -1543,10 +1558,10 @@
         <v>5</v>
       </c>
       <c r="L25">
-        <v>0.02652654238045216</v>
+        <v>0.01511699799448252</v>
       </c>
       <c r="M25">
-        <v>0.05044718086719513</v>
+        <v>0.2268946468830109</v>
       </c>
     </row>
     <row r="26" spans="1:13">
@@ -1554,19 +1569,19 @@
         <v>37</v>
       </c>
       <c r="B26">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C26">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D26">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
       <c r="F26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G26">
         <v>1</v>
@@ -1575,7 +1590,7 @@
         <v>2e-07</v>
       </c>
       <c r="I26">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="J26">
         <v>8</v>
@@ -1584,10 +1599,10 @@
         <v>5</v>
       </c>
       <c r="L26">
-        <v>0.0144530413672328</v>
+        <v>0.0137598505243659</v>
       </c>
       <c r="M26">
-        <v>0.2646083831787109</v>
+        <v>0.2512792944908142</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -1595,28 +1610,28 @@
         <v>38</v>
       </c>
       <c r="B27">
+        <v>5</v>
+      </c>
+      <c r="C27">
+        <v>16</v>
+      </c>
+      <c r="D27">
+        <v>16</v>
+      </c>
+      <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
         <v>3</v>
       </c>
-      <c r="C27">
-        <v>8</v>
-      </c>
-      <c r="D27">
-        <v>32</v>
-      </c>
-      <c r="E27">
-        <v>1</v>
-      </c>
-      <c r="F27">
-        <v>2</v>
-      </c>
       <c r="G27">
         <v>1</v>
       </c>
       <c r="H27">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I27">
-        <v>0.0007</v>
+        <v>0.0001</v>
       </c>
       <c r="J27">
         <v>8</v>
@@ -1625,10 +1640,10 @@
         <v>5</v>
       </c>
       <c r="L27">
-        <v>0.01031966041773558</v>
+        <v>0.01508545223623514</v>
       </c>
       <c r="M27">
-        <v>0.3306339383125305</v>
+        <v>0.2195451408624649</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -1639,7 +1654,7 @@
         <v>3</v>
       </c>
       <c r="C28">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D28">
         <v>16</v>
@@ -1654,10 +1669,10 @@
         <v>1</v>
       </c>
       <c r="H28">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I28">
-        <v>0.0007</v>
+        <v>0.0001</v>
       </c>
       <c r="J28">
         <v>8</v>
@@ -1666,10 +1681,10 @@
         <v>5</v>
       </c>
       <c r="L28">
-        <v>0.009471160359680653</v>
+        <v>0.01565391197800636</v>
       </c>
       <c r="M28">
-        <v>0.3517069518566132</v>
+        <v>0.2294184565544128</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -1680,7 +1695,7 @@
         <v>3</v>
       </c>
       <c r="C29">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="D29">
         <v>32</v>
@@ -1695,10 +1710,10 @@
         <v>1</v>
       </c>
       <c r="H29">
-        <v>2e-07</v>
+        <v>5e-07</v>
       </c>
       <c r="I29">
-        <v>0.0007</v>
+        <v>6.999999999999999e-05</v>
       </c>
       <c r="J29">
         <v>8</v>
@@ -1707,10 +1722,10 @@
         <v>5</v>
       </c>
       <c r="L29">
-        <v>0.008939820341765881</v>
+        <v>0.01425743196159601</v>
       </c>
       <c r="M29">
-        <v>0.35904461145401</v>
+        <v>0.2467455416917801</v>
       </c>
     </row>
     <row r="30" spans="1:13">
@@ -1721,7 +1736,7 @@
         <v>3</v>
       </c>
       <c r="C30">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D30">
         <v>16</v>
@@ -1736,10 +1751,10 @@
         <v>1</v>
       </c>
       <c r="H30">
-        <v>2e-07</v>
+        <v>2e-06</v>
       </c>
       <c r="I30">
-        <v>0.0007</v>
+        <v>0.001</v>
       </c>
       <c r="J30">
         <v>8</v>
@@ -1748,10 +1763,10 @@
         <v>5</v>
       </c>
       <c r="L30">
-        <v>0.01335400622338057</v>
+        <v>0.01414524763822556</v>
       </c>
       <c r="M30">
-        <v>0.2640894949436188</v>
+        <v>0.2320943474769592</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -1762,25 +1777,25 @@
         <v>3</v>
       </c>
       <c r="C31">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D31">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E31">
         <v>1</v>
       </c>
       <c r="F31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G31">
         <v>1</v>
       </c>
       <c r="H31">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I31">
-        <v>0.0007</v>
+        <v>0.00015</v>
       </c>
       <c r="J31">
         <v>8</v>
@@ -1789,10 +1804,10 @@
         <v>5</v>
       </c>
       <c r="L31">
-        <v>0.02298250235617161</v>
+        <v>0.01530452910810709</v>
       </c>
       <c r="M31">
-        <v>0.08047252893447876</v>
+        <v>0.2169028967618942</v>
       </c>
     </row>
     <row r="32" spans="1:13">
@@ -1800,10 +1815,10 @@
         <v>43</v>
       </c>
       <c r="B32">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C32">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D32">
         <v>16</v>
@@ -1812,16 +1827,16 @@
         <v>1</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G32">
         <v>1</v>
       </c>
       <c r="H32">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I32">
-        <v>0.0007</v>
+        <v>0.0008</v>
       </c>
       <c r="J32">
         <v>8</v>
@@ -1830,10 +1845,10 @@
         <v>5</v>
       </c>
       <c r="L32">
-        <v>0.005876542069017887</v>
+        <v>0.01104966644197702</v>
       </c>
       <c r="M32">
-        <v>0.3449607789516449</v>
+        <v>0.3225390315055847</v>
       </c>
     </row>
     <row r="33" spans="1:13">
@@ -1841,28 +1856,28 @@
         <v>44</v>
       </c>
       <c r="B33">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C33">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D33">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E33">
         <v>1</v>
       </c>
       <c r="F33">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G33">
         <v>1</v>
       </c>
       <c r="H33">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I33">
-        <v>0.0007</v>
+        <v>2.5e-05</v>
       </c>
       <c r="J33">
         <v>8</v>
@@ -1871,10 +1886,10 @@
         <v>5</v>
       </c>
       <c r="L33">
-        <v>0.01197956781834364</v>
+        <v>0.01682636886835098</v>
       </c>
       <c r="M33">
-        <v>0.2813169360160828</v>
+        <v>0.1849002987146378</v>
       </c>
     </row>
     <row r="34" spans="1:13">
@@ -1885,7 +1900,7 @@
         <v>6</v>
       </c>
       <c r="C34">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D34">
         <v>16</v>
@@ -1894,16 +1909,16 @@
         <v>1</v>
       </c>
       <c r="F34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G34">
         <v>1</v>
       </c>
       <c r="H34">
-        <v>2e-07</v>
+        <v>1e-06</v>
       </c>
       <c r="I34">
-        <v>0.0007</v>
+        <v>8.000000000000001e-05</v>
       </c>
       <c r="J34">
         <v>8</v>
@@ -1912,10 +1927,10 @@
         <v>5</v>
       </c>
       <c r="L34">
-        <v>0.01171945314854383</v>
+        <v>0.0153689356520772</v>
       </c>
       <c r="M34">
-        <v>0.3067871332168579</v>
+        <v>0.2342420518398285</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -1923,19 +1938,19 @@
         <v>46</v>
       </c>
       <c r="B35">
+        <v>6</v>
+      </c>
+      <c r="C35">
+        <v>32</v>
+      </c>
+      <c r="D35">
+        <v>32</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
         <v>2</v>
-      </c>
-      <c r="C35">
-        <v>8</v>
-      </c>
-      <c r="D35">
-        <v>16</v>
-      </c>
-      <c r="E35">
-        <v>1</v>
-      </c>
-      <c r="F35">
-        <v>4</v>
       </c>
       <c r="G35">
         <v>1</v>
@@ -1944,7 +1959,7 @@
         <v>2e-07</v>
       </c>
       <c r="I35">
-        <v>0.0007</v>
+        <v>0.0001</v>
       </c>
       <c r="J35">
         <v>8</v>
@@ -1953,10 +1968,10 @@
         <v>5</v>
       </c>
       <c r="L35">
-        <v>0.02075445093214512</v>
+        <v>0.01123293489217758</v>
       </c>
       <c r="M35">
-        <v>0.1012341752648354</v>
+        <v>0.3346756100654602</v>
       </c>
     </row>
     <row r="36" spans="1:13">
@@ -1964,10 +1979,10 @@
         <v>47</v>
       </c>
       <c r="B36">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C36">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D36">
         <v>16</v>
@@ -1976,16 +1991,16 @@
         <v>1</v>
       </c>
       <c r="F36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G36">
         <v>1</v>
       </c>
       <c r="H36">
-        <v>2e-07</v>
+        <v>2e-06</v>
       </c>
       <c r="I36">
-        <v>0.0007</v>
+        <v>6e-05</v>
       </c>
       <c r="J36">
         <v>8</v>
@@ -1994,10 +2009,10 @@
         <v>5</v>
       </c>
       <c r="L36">
-        <v>0.01198610290884972</v>
+        <v>0.01943289116024971</v>
       </c>
       <c r="M36">
-        <v>0.2936770021915436</v>
+        <v>0.1891117542982101</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -2005,13 +2020,13 @@
         <v>48</v>
       </c>
       <c r="B37">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C37">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="D37">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -2026,7 +2041,7 @@
         <v>2e-07</v>
       </c>
       <c r="I37">
-        <v>0.0007</v>
+        <v>3e-05</v>
       </c>
       <c r="J37">
         <v>8</v>
@@ -2035,10 +2050,10 @@
         <v>5</v>
       </c>
       <c r="L37">
-        <v>0.01439808961004019</v>
+        <v>0.01914861612021923</v>
       </c>
       <c r="M37">
-        <v>0.2381373792886734</v>
+        <v>0.1948999911546707</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -2049,7 +2064,7 @@
         <v>2</v>
       </c>
       <c r="C38">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D38">
         <v>16</v>
@@ -2058,28 +2073,233 @@
         <v>1</v>
       </c>
       <c r="F38">
+        <v>2</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="H38">
+        <v>2e-06</v>
+      </c>
+      <c r="I38">
+        <v>0.0001</v>
+      </c>
+      <c r="J38">
+        <v>8</v>
+      </c>
+      <c r="K38">
+        <v>5</v>
+      </c>
+      <c r="L38">
+        <v>0.01701854541897774</v>
+      </c>
+      <c r="M38">
+        <v>0.1944358199834824</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13">
+      <c r="A39" t="s">
+        <v>50</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39">
+        <v>32</v>
+      </c>
+      <c r="D39">
+        <v>32</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
+        <v>2</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>1e-06</v>
+      </c>
+      <c r="I39">
+        <v>0.00025</v>
+      </c>
+      <c r="J39">
+        <v>8</v>
+      </c>
+      <c r="K39">
+        <v>5</v>
+      </c>
+      <c r="L39">
+        <v>0.01302684843540192</v>
+      </c>
+      <c r="M39">
+        <v>0.280820369720459</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13">
+      <c r="A40" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40">
+        <v>2</v>
+      </c>
+      <c r="C40">
+        <v>16</v>
+      </c>
+      <c r="D40">
+        <v>16</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40">
+        <v>6e-06</v>
+      </c>
+      <c r="I40">
+        <v>0.0002</v>
+      </c>
+      <c r="J40">
+        <v>8</v>
+      </c>
+      <c r="K40">
+        <v>5</v>
+      </c>
+      <c r="L40">
+        <v>0.01696995086967945</v>
+      </c>
+      <c r="M40">
+        <v>0.1820677667856216</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13">
+      <c r="A41" t="s">
+        <v>52</v>
+      </c>
+      <c r="B41">
+        <v>2</v>
+      </c>
+      <c r="C41">
+        <v>32</v>
+      </c>
+      <c r="D41">
+        <v>32</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="H41">
+        <v>1e-06</v>
+      </c>
+      <c r="I41">
+        <v>0.001</v>
+      </c>
+      <c r="J41">
+        <v>8</v>
+      </c>
+      <c r="K41">
+        <v>5</v>
+      </c>
+      <c r="L41">
+        <v>0.01382499188184738</v>
+      </c>
+      <c r="M41">
+        <v>0.2490603476762772</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13">
+      <c r="A42" t="s">
+        <v>53</v>
+      </c>
+      <c r="B42">
+        <v>2</v>
+      </c>
+      <c r="C42">
+        <v>16</v>
+      </c>
+      <c r="D42">
+        <v>16</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42">
         <v>3</v>
       </c>
-      <c r="G38">
-        <v>1</v>
-      </c>
-      <c r="H38">
-        <v>2e-07</v>
-      </c>
-      <c r="I38">
-        <v>0.0007</v>
-      </c>
-      <c r="J38">
-        <v>8</v>
-      </c>
-      <c r="K38">
-        <v>5</v>
-      </c>
-      <c r="L38">
-        <v>0.01031064987182617</v>
-      </c>
-      <c r="M38">
-        <v>0.3455671370029449</v>
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>1.7e-06</v>
+      </c>
+      <c r="I42">
+        <v>5e-05</v>
+      </c>
+      <c r="J42">
+        <v>8</v>
+      </c>
+      <c r="K42">
+        <v>5</v>
+      </c>
+      <c r="L42">
+        <v>0.01932175830006599</v>
+      </c>
+      <c r="M42">
+        <v>0.1461078226566315</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13">
+      <c r="A43" t="s">
+        <v>54</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43">
+        <v>32</v>
+      </c>
+      <c r="D43">
+        <v>32</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
+        <v>3</v>
+      </c>
+      <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="H43">
+        <v>1e-06</v>
+      </c>
+      <c r="I43">
+        <v>4e-05</v>
+      </c>
+      <c r="J43">
+        <v>8</v>
+      </c>
+      <c r="K43">
+        <v>5</v>
+      </c>
+      <c r="L43">
+        <v>0.01711563393473625</v>
+      </c>
+      <c r="M43">
+        <v>0.1867019683122635</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ensure output excel path is defined
</commit_message>
<xml_diff>
--- a/Deep_Learning/Model_Optimization.xlsx
+++ b/Deep_Learning/Model_Optimization.xlsx
@@ -697,10 +697,10 @@
         <v>5</v>
       </c>
       <c r="L4">
-        <v>0.01579839736223221</v>
+        <v>0.01503736805170774</v>
       </c>
       <c r="M4">
-        <v>0.2252430766820908</v>
+        <v>0.237884521484375</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -741,7 +741,7 @@
         <v>0.0230035912245512</v>
       </c>
       <c r="M5">
-        <v>0.1652709096670151</v>
+        <v>0.1798733919858932</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -823,7 +823,7 @@
         <v>0.01491123158484697</v>
       </c>
       <c r="M7">
-        <v>0.2240881472826004</v>
+        <v>0.2283452153205872</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -943,7 +943,7 @@
         <v>5</v>
       </c>
       <c r="L10">
-        <v>0.01578664220869541</v>
+        <v>0.01575510948896408</v>
       </c>
       <c r="M10">
         <v>0.2078990191221237</v>
@@ -987,7 +987,7 @@
         <v>0.01563869044184685</v>
       </c>
       <c r="M11">
-        <v>0.1988261938095093</v>
+        <v>0.2002087831497192</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1025,10 +1025,10 @@
         <v>5</v>
       </c>
       <c r="L12">
-        <v>0.01966289430856705</v>
+        <v>0.01939504779875278</v>
       </c>
       <c r="M12">
-        <v>0.1412597149610519</v>
+        <v>0.1515783220529556</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1066,10 +1066,10 @@
         <v>5</v>
       </c>
       <c r="L13">
-        <v>0.01759837009012699</v>
+        <v>0.01727837882936001</v>
       </c>
       <c r="M13">
-        <v>0.1507639437913895</v>
+        <v>0.18096724152565</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -1189,10 +1189,10 @@
         <v>5</v>
       </c>
       <c r="L16">
-        <v>0.01620516367256641</v>
+        <v>0.01517524290829897</v>
       </c>
       <c r="M16">
-        <v>0.2279257923364639</v>
+        <v>0.2407675981521606</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1230,7 +1230,7 @@
         <v>5</v>
       </c>
       <c r="L17">
-        <v>0.0195910632610321</v>
+        <v>0.01832686737179756</v>
       </c>
       <c r="M17">
         <v>0.2124533653259277</v>
@@ -1394,10 +1394,10 @@
         <v>5</v>
       </c>
       <c r="L21">
-        <v>0.01484843157231808</v>
+        <v>0.01416316721588373</v>
       </c>
       <c r="M21">
-        <v>0.2374653369188309</v>
+        <v>0.2390248328447342</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1435,10 +1435,10 @@
         <v>5</v>
       </c>
       <c r="L22">
-        <v>0.01789148151874542</v>
+        <v>0.01683954522013664</v>
       </c>
       <c r="M22">
-        <v>0.1609459668397903</v>
+        <v>0.1937897652387619</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1476,10 +1476,10 @@
         <v>5</v>
       </c>
       <c r="L23">
-        <v>0.01326036639511585</v>
+        <v>0.01194720901548862</v>
       </c>
       <c r="M23">
-        <v>0.2676254212856293</v>
+        <v>0.2966634929180145</v>
       </c>
     </row>
     <row r="24" spans="1:13">
@@ -1517,10 +1517,10 @@
         <v>5</v>
       </c>
       <c r="L24">
-        <v>0.01356085110455751</v>
+        <v>0.01310379803180695</v>
       </c>
       <c r="M24">
-        <v>0.2645507454872131</v>
+        <v>0.2703265845775604</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -1599,10 +1599,10 @@
         <v>5</v>
       </c>
       <c r="L26">
-        <v>0.0137598505243659</v>
+        <v>0.01360708475112915</v>
       </c>
       <c r="M26">
-        <v>0.2512792944908142</v>
+        <v>0.2633950114250183</v>
       </c>
     </row>
     <row r="27" spans="1:13">
@@ -1722,7 +1722,7 @@
         <v>5</v>
       </c>
       <c r="L29">
-        <v>0.01425743196159601</v>
+        <v>0.01422695629298687</v>
       </c>
       <c r="M29">
         <v>0.2467455416917801</v>
@@ -1766,7 +1766,7 @@
         <v>0.01414524763822556</v>
       </c>
       <c r="M30">
-        <v>0.2320943474769592</v>
+        <v>0.239423468708992</v>
       </c>
     </row>
     <row r="31" spans="1:13">
@@ -1927,10 +1927,10 @@
         <v>5</v>
       </c>
       <c r="L34">
-        <v>0.0153689356520772</v>
+        <v>0.013644739985466</v>
       </c>
       <c r="M34">
-        <v>0.2342420518398285</v>
+        <v>0.258403092622757</v>
       </c>
     </row>
     <row r="35" spans="1:13">
@@ -1968,7 +1968,7 @@
         <v>5</v>
       </c>
       <c r="L35">
-        <v>0.01123293489217758</v>
+        <v>0.01087185554206371</v>
       </c>
       <c r="M35">
         <v>0.3346756100654602</v>
@@ -2009,10 +2009,10 @@
         <v>5</v>
       </c>
       <c r="L36">
-        <v>0.01943289116024971</v>
+        <v>0.01821470260620117</v>
       </c>
       <c r="M36">
-        <v>0.1891117542982101</v>
+        <v>0.2004352211952209</v>
       </c>
     </row>
     <row r="37" spans="1:13">
@@ -2050,10 +2050,10 @@
         <v>5</v>
       </c>
       <c r="L37">
-        <v>0.01914861612021923</v>
+        <v>0.01854624226689339</v>
       </c>
       <c r="M37">
-        <v>0.1948999911546707</v>
+        <v>0.20271235704422</v>
       </c>
     </row>
     <row r="38" spans="1:13">
@@ -2091,10 +2091,10 @@
         <v>5</v>
       </c>
       <c r="L38">
-        <v>0.01701854541897774</v>
+        <v>0.01659020595252514</v>
       </c>
       <c r="M38">
-        <v>0.1944358199834824</v>
+        <v>0.2046237736940384</v>
       </c>
     </row>
     <row r="39" spans="1:13">
@@ -2132,10 +2132,10 @@
         <v>5</v>
       </c>
       <c r="L39">
-        <v>0.01302684843540192</v>
+        <v>0.01153793837875128</v>
       </c>
       <c r="M39">
-        <v>0.280820369720459</v>
+        <v>0.3045293092727661</v>
       </c>
     </row>
     <row r="40" spans="1:13">
@@ -2173,10 +2173,10 @@
         <v>5</v>
       </c>
       <c r="L40">
-        <v>0.01696995086967945</v>
+        <v>0.01662307046353817</v>
       </c>
       <c r="M40">
-        <v>0.1820677667856216</v>
+        <v>0.1868326365947723</v>
       </c>
     </row>
     <row r="41" spans="1:13">
@@ -2299,7 +2299,7 @@
         <v>0.01711563393473625</v>
       </c>
       <c r="M43">
-        <v>0.1867019683122635</v>
+        <v>0.1877612322568893</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
found best loss to be 4 layers, 8 filters, 32 max. Running with different step_size factors for a factor of 10 epochs + 1
</commit_message>
<xml_diff>
--- a/Deep_Learning/Model_Optimization.xlsx
+++ b/Deep_Learning/Model_Optimization.xlsx
@@ -358,7 +358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -425,10 +425,10 @@
         <v>0.001</v>
       </c>
       <c r="G2" t="n">
-        <v>0.01324630063027143</v>
+        <v>0.01543555036187172</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3500925898551941</v>
+        <v>0.3027568161487579</v>
       </c>
     </row>
     <row r="3">
@@ -453,16 +453,16 @@
         <v>0.001</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0128286499530077</v>
+        <v>0.01422119978815317</v>
       </c>
       <c r="H3" t="n">
-        <v>0.3439555466175079</v>
+        <v>0.3143450617790222</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>1layers16filters32max_filters8e-06min_lr0.001max_lr</t>
+          <t>1layers16filters32max_filters8e-06min_lr0.0008max_lr</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -478,13 +478,13 @@
         <v>8e-06</v>
       </c>
       <c r="F4" t="n">
-        <v>0.001</v>
+        <v>0.0008</v>
       </c>
       <c r="G4" t="n">
-        <v>0.01275630109012127</v>
+        <v>0.01433329377323389</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3692083656787872</v>
+        <v>0.3115420341491699</v>
       </c>
     </row>
     <row r="5">
@@ -509,20 +509,20 @@
         <v>0.0008</v>
       </c>
       <c r="G5" t="n">
-        <v>0.01314476598054171</v>
+        <v>0.01505056116729975</v>
       </c>
       <c r="H5" t="n">
-        <v>0.360489159822464</v>
+        <v>0.3276698291301727</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>3layers8filters32max_filters4e-06min_lr0.0005max_lr</t>
+          <t>4layers8filters32max_filters1e-06min_lr0.0002max_lr</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
         <v>8</v>
@@ -531,26 +531,26 @@
         <v>32</v>
       </c>
       <c r="E6" t="n">
-        <v>4e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0005</v>
+        <v>0.0002</v>
       </c>
       <c r="G6" t="n">
-        <v>0.008851006627082825</v>
+        <v>0.01184713374823332</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4835479855537415</v>
+        <v>0.3803465068340302</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3layers8filters16max_filters4e-06min_lr0.0005max_lr</t>
+          <t>4layers8filters16max_filters1e-06min_lr0.00013max_lr</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
         <v>8</v>
@@ -559,26 +559,26 @@
         <v>16</v>
       </c>
       <c r="E7" t="n">
-        <v>4e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0005</v>
+        <v>0.00013</v>
       </c>
       <c r="G7" t="n">
-        <v>0.009349489584565163</v>
+        <v>0.01367784384638071</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4581268727779388</v>
+        <v>0.3203473389148712</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>3layers16filters32max_filters3e-06min_lr0.0001max_lr</t>
+          <t>4layers16filters32max_filters2e-06min_lr0.0001max_lr</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C8" t="n">
         <v>16</v>
@@ -587,26 +587,26 @@
         <v>32</v>
       </c>
       <c r="E8" t="n">
-        <v>3e-06</v>
+        <v>2e-06</v>
       </c>
       <c r="F8" t="n">
         <v>0.0001</v>
       </c>
       <c r="G8" t="n">
-        <v>0.01141284126788378</v>
+        <v>0.01269377488642931</v>
       </c>
       <c r="H8" t="n">
-        <v>0.3835093379020691</v>
+        <v>0.3423174023628235</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3layers16filters16max_filters4e-06min_lr0.0003max_lr</t>
+          <t>4layers16filters16max_filters2e-06min_lr0.0001max_lr</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
         <v>16</v>
@@ -615,26 +615,26 @@
         <v>16</v>
       </c>
       <c r="E9" t="n">
-        <v>4e-06</v>
+        <v>2e-06</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0003</v>
+        <v>0.0001</v>
       </c>
       <c r="G9" t="n">
-        <v>0.009973978623747826</v>
+        <v>0.01423004176467657</v>
       </c>
       <c r="H9" t="n">
-        <v>0.4378767609596252</v>
+        <v>0.3225606083869934</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2layers8filters32max_filters8e-06min_lr0.0008max_lr</t>
+          <t>5layers8filters32max_filters1e-06min_lr0.0001max_lr</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C10" t="n">
         <v>8</v>
@@ -643,26 +643,26 @@
         <v>32</v>
       </c>
       <c r="E10" t="n">
-        <v>8e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0008</v>
+        <v>0.0001</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01048335991799831</v>
+        <v>0.01314619649201632</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4118861854076385</v>
+        <v>0.3471824824810028</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2layers8filters16max_filters8e-06min_lr0.0008max_lr</t>
+          <t>5layers8filters16max_filters1e-06min_lr0.0001max_lr</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C11" t="n">
         <v>8</v>
@@ -671,26 +671,26 @@
         <v>16</v>
       </c>
       <c r="E11" t="n">
-        <v>8e-06</v>
+        <v>1e-06</v>
       </c>
       <c r="F11" t="n">
-        <v>0.0008</v>
+        <v>0.0001</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01078045926988125</v>
+        <v>0.01296063605695963</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4092032909393311</v>
+        <v>0.329539567232132</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2layers16filters32max_filters1e-06min_lr0.0004max_lr</t>
+          <t>5layers16filters32max_filters1e-06min_lr2e-05max_lr</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C12" t="n">
         <v>16</v>
@@ -702,41 +702,265 @@
         <v>1e-06</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0004</v>
+        <v>2e-05</v>
       </c>
       <c r="G12" t="n">
-        <v>0.009933600202202797</v>
+        <v>0.01671410724520683</v>
       </c>
       <c r="H12" t="n">
-        <v>0.4357804358005524</v>
+        <v>0.2684630751609802</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2layers16filters16max_filters1e-06min_lr0.0004max_lr</t>
+          <t>5layers16filters16max_filters1e-06min_lr0.0001max_lr</t>
         </is>
       </c>
       <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>16</v>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.01344846468418837</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.307561069726944</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>3layers8filters32max_filters1e-06min_lr6e-05max_lr</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" t="n">
+        <v>8</v>
+      </c>
+      <c r="D14" t="n">
+        <v>32</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6e-05</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.0150853730738163</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.2726874053478241</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>3layers8filters16max_filters5e-06min_lr0.0002max_lr</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>8</v>
+      </c>
+      <c r="D15" t="n">
+        <v>16</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5e-06</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.01356527395546436</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3157221674919128</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>3layers16filters32max_filters1e-06min_lr8e-05max_lr</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="n">
+        <v>16</v>
+      </c>
+      <c r="D16" t="n">
+        <v>32</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8.000000000000001e-05</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.01363150030374527</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.3109259903430939</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>3layers16filters16max_filters4e-06min_lr0.0001max_lr</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="n">
+        <v>16</v>
+      </c>
+      <c r="D17" t="n">
+        <v>16</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4e-06</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.0145391495898366</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.291810005903244</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2layers8filters32max_filters1e-06min_lr0.0008max_lr</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>2</v>
       </c>
-      <c r="C13" t="n">
-        <v>16</v>
-      </c>
-      <c r="D13" t="n">
-        <v>16</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1e-06</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0.01052340772002935</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.4182655513286591</v>
+      <c r="C18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D18" t="n">
+        <v>32</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.01344506721943617</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.3427440822124481</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2layers8filters16max_filters8e-06min_lr0.0006max_lr</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>8</v>
+      </c>
+      <c r="D19" t="n">
+        <v>16</v>
+      </c>
+      <c r="E19" t="n">
+        <v>8e-06</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.0135336983948946</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.3135663568973541</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2layers16filters32max_filters1e-06min_lr0.0002max_lr</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
+        <v>16</v>
+      </c>
+      <c r="D20" t="n">
+        <v>32</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.01351331640034914</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.329128235578537</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2layers16filters16max_filters1e-06min_lr0.0003max_lr</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>16</v>
+      </c>
+      <c r="D21" t="n">
+        <v>16</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1e-06</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.01437020860612392</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.3183757960796356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>